<commit_message>
thêm vat, phí shipp, phí khác khi tạo đơn hàng
</commit_message>
<xml_diff>
--- a/public/files/import/template_products_update_inventory.xlsx
+++ b/public/files/import/template_products_update_inventory.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E066FE-DF35-4B2C-B2B7-A93A565337EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A76F59-6D1E-4433-98B8-00CA30E156FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Mã sản phẩm</t>
   </si>
@@ -40,31 +40,34 @@
     <t>SL: Sản Xuất</t>
   </si>
   <si>
-    <t>sp04</t>
+    <t>SP001</t>
+  </si>
+  <si>
+    <t>Sản phẩm 01</t>
+  </si>
+  <si>
+    <t>SP002</t>
+  </si>
+  <si>
+    <t>Sản phẩm 02</t>
+  </si>
+  <si>
+    <t>SP003</t>
+  </si>
+  <si>
+    <t>Sản phẩm 03</t>
+  </si>
+  <si>
+    <t>SP004</t>
   </si>
   <si>
     <t>Sản phẩm 04</t>
   </si>
   <si>
-    <t>sp02</t>
-  </si>
-  <si>
-    <t>sản phẩm 2</t>
-  </si>
-  <si>
-    <t>SP03</t>
-  </si>
-  <si>
-    <t>Thảm da cao cấp</t>
-  </si>
-  <si>
-    <t>SP01</t>
-  </si>
-  <si>
-    <t>SP10</t>
-  </si>
-  <si>
-    <t>Thảm sàn nhựa đúc VF3</t>
+    <t>SP005</t>
+  </si>
+  <si>
+    <t>Sản phẩm 05</t>
   </si>
 </sst>
 </file>
@@ -415,7 +418,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
@@ -453,13 +456,13 @@
         <v>10</v>
       </c>
       <c r="D2">
+        <v>9</v>
+      </c>
+      <c r="E2">
+        <v>19</v>
+      </c>
+      <c r="F2">
         <v>20</v>
-      </c>
-      <c r="E2">
-        <v>30</v>
-      </c>
-      <c r="F2">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -470,16 +473,16 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E3">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F3">
-        <v>42</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -490,16 +493,16 @@
         <v>11</v>
       </c>
       <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>12</v>
+      </c>
+      <c r="E4">
         <v>14</v>
       </c>
-      <c r="D4">
-        <v>24</v>
-      </c>
-      <c r="E4">
-        <v>34</v>
-      </c>
       <c r="F4">
-        <v>44</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -507,39 +510,39 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+      <c r="D5">
         <v>11</v>
       </c>
-      <c r="C5">
-        <v>16</v>
-      </c>
-      <c r="D5">
-        <v>26</v>
-      </c>
       <c r="E5">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F5">
-        <v>46</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
         <v>14</v>
       </c>
-      <c r="C6">
-        <v>18</v>
-      </c>
-      <c r="D6">
-        <v>28</v>
-      </c>
-      <c r="E6">
-        <v>38</v>
-      </c>
       <c r="F6">
-        <v>48</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cập nhật tồn kho sản phẩm theo từng kho
</commit_message>
<xml_diff>
--- a/public/files/import/template_products_update_inventory.xlsx
+++ b/public/files/import/template_products_update_inventory.xlsx
@@ -1,26 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14A76F59-6D1E-4433-98B8-00CA30E156FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>Mã sản phẩm</t>
   </si>
@@ -37,51 +32,56 @@
     <t>SL: Kho Hồ Chí Minh</t>
   </si>
   <si>
-    <t>SL: Sản Xuất</t>
-  </si>
-  <si>
-    <t>SP001</t>
-  </si>
-  <si>
-    <t>Sản phẩm 01</t>
-  </si>
-  <si>
-    <t>SP002</t>
-  </si>
-  <si>
-    <t>Sản phẩm 02</t>
-  </si>
-  <si>
-    <t>SP003</t>
-  </si>
-  <si>
-    <t>Sản phẩm 03</t>
-  </si>
-  <si>
-    <t>SP004</t>
-  </si>
-  <si>
-    <t>Sản phẩm 04</t>
-  </si>
-  <si>
-    <t>SP005</t>
-  </si>
-  <si>
-    <t>Sản phẩm 05</t>
+    <t>khanlau</t>
+  </si>
+  <si>
+    <t>Khăn Lau</t>
+  </si>
+  <si>
+    <t>bangdinh</t>
+  </si>
+  <si>
+    <t>Phu Kiện Băng Dính</t>
+  </si>
+  <si>
+    <t>chotroi</t>
+  </si>
+  <si>
+    <t>Phu Kiện Chốt Rối</t>
+  </si>
+  <si>
+    <t>COP-033</t>
+  </si>
+  <si>
+    <t>Thảm Cốp Nhựa Đúc PAKO 2008 18 - 25</t>
+  </si>
+  <si>
+    <t>COP-024</t>
+  </si>
+  <si>
+    <t>Thảm Cốp Nhựa Đúc PAKO BYD Sealion 6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -92,38 +92,31 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -413,19 +406,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.996582" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="43.560791" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="21.137695" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="17.567139" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="23.422852" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -441,112 +436,104 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>775</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2">
+        <v>84</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="C2">
-        <v>10</v>
-      </c>
-      <c r="D2">
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3">
         <v>9</v>
-      </c>
-      <c r="E2">
-        <v>19</v>
-      </c>
-      <c r="F2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
       </c>
       <c r="D3">
         <v>10</v>
       </c>
       <c r="E3">
-        <v>23</v>
-      </c>
-      <c r="F3">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-      <c r="D4">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="E4">
+      <c r="C5">
+        <v>1000</v>
+      </c>
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="F4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5">
-        <v>10</v>
-      </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>14</v>
-      </c>
-      <c r="F5">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
       <c r="C6">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="E6">
-        <v>14</v>
-      </c>
-      <c r="F6">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>